<commit_message>
feat: update study set handling in AbstractHierarchicalImportService and clean up ScheduleModuleType and AvailableScheduleModule components
</commit_message>
<xml_diff>
--- a/repo-writing/test-data/writing-import-chinese-standard.xlsx
+++ b/repo-writing/test-data/writing-import-chinese-standard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DO_AN\BE_LMS\repo-writing\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B36A8058-A8C2-4B44-82CA-0421DE80E907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AACB6005-061D-4ABA-AE90-76A77735D6E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -561,7 +561,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T15"/>
+  <dimension ref="A1:T9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
@@ -803,8 +803,8 @@
         <v>63</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="S15" t="s">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="S9" t="s">
         <v>64</v>
       </c>
     </row>

</xml_diff>